<commit_message>
feat: add Nodemailer Gmail SMTP support & workflow secrets
</commit_message>
<xml_diff>
--- a/data/applications_tracker.xlsx
+++ b/data/applications_tracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L36"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -453,7 +453,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>app_1790009309416_0</v>
+        <v>app_1790010835509_0</v>
       </c>
       <c r="B2" t="str">
         <v>Palo Alto Networks</v>
@@ -480,7 +480,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.509Z</v>
       </c>
       <c r="K2" t="str">
         <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
@@ -491,7 +491,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>app_1790009309416_1</v>
+        <v>app_1790010835509_1</v>
       </c>
       <c r="B3" t="str">
         <v>CrowdStrike</v>
@@ -518,7 +518,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.509Z</v>
       </c>
       <c r="K3" t="str">
         <v>https://crowdstrike.com/careers/ai-security-specialist</v>
@@ -529,7 +529,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>app_1790009309416_2</v>
+        <v>app_1790010835510_2</v>
       </c>
       <c r="B4" t="str">
         <v>Darktrace</v>
@@ -556,7 +556,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K4" t="str">
         <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>app_1790009309417_3</v>
+        <v>app_1790010835510_3</v>
       </c>
       <c r="B5" t="str">
         <v>Cloudflare</v>
@@ -594,7 +594,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-09-21T16:48:29.417Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K5" t="str">
         <v>https://cloudflare.com/careers/security-automation</v>
@@ -605,7 +605,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>app_1790009309417_4</v>
+        <v>app_1790010835510_4</v>
       </c>
       <c r="B6" t="str">
         <v>Anthropic</v>
@@ -632,7 +632,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-09-21T16:48:29.417Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K6" t="str">
         <v>https://anthropic.com/careers/fullstack-ai-security</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>app_1790009257131_0</v>
+        <v>app_1790009309416_0</v>
       </c>
       <c r="B7" t="str">
         <v>Palo Alto Networks</v>
@@ -658,30 +658,30 @@
         <v>Greenhouse</v>
       </c>
       <c r="F7" t="str">
-        <v>61%</v>
+        <v>92%</v>
       </c>
       <c r="G7" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H7" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I7" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K7" t="str">
         <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
       </c>
       <c r="L7" t="str">
-        <v>Skipped: Match score 61% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>app_1790009257131_1</v>
+        <v>app_1790009309416_1</v>
       </c>
       <c r="B8" t="str">
         <v>CrowdStrike</v>
@@ -696,30 +696,30 @@
         <v>Lever</v>
       </c>
       <c r="F8" t="str">
-        <v>61%</v>
+        <v>92%</v>
       </c>
       <c r="G8" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H8" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I8" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K8" t="str">
         <v>https://crowdstrike.com/careers/ai-security-specialist</v>
       </c>
       <c r="L8" t="str">
-        <v>Skipped: Match score 61% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>app_1790009257131_2</v>
+        <v>app_1790009309416_2</v>
       </c>
       <c r="B9" t="str">
         <v>Darktrace</v>
@@ -734,30 +734,30 @@
         <v>Greenhouse</v>
       </c>
       <c r="F9" t="str">
-        <v>50%</v>
+        <v>74%</v>
       </c>
       <c r="G9" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H9" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I9" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J9" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K9" t="str">
         <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
       </c>
       <c r="L9" t="str">
-        <v>Skipped: Match score 50% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>app_1790009257131_3</v>
+        <v>app_1790009309417_3</v>
       </c>
       <c r="B10" t="str">
         <v>Cloudflare</v>
@@ -772,30 +772,30 @@
         <v>Workday</v>
       </c>
       <c r="F10" t="str">
-        <v>51%</v>
+        <v>90%</v>
       </c>
       <c r="G10" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H10" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I10" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J10" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.417Z</v>
       </c>
       <c r="K10" t="str">
         <v>https://cloudflare.com/careers/security-automation</v>
       </c>
       <c r="L10" t="str">
-        <v>Skipped: Match score 51% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>app_1790009257131_4</v>
+        <v>app_1790009309417_4</v>
       </c>
       <c r="B11" t="str">
         <v>Anthropic</v>
@@ -810,45 +810,45 @@
         <v>Greenhouse</v>
       </c>
       <c r="F11" t="str">
-        <v>50%</v>
+        <v>74%</v>
       </c>
       <c r="G11" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H11" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I11" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J11" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.417Z</v>
       </c>
       <c r="K11" t="str">
         <v>https://anthropic.com/careers/fullstack-ai-security</v>
       </c>
       <c r="L11" t="str">
-        <v>Skipped: Match score 50% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>app_1790008945002_0</v>
+        <v>app_1790009257131_0</v>
       </c>
       <c r="B12" t="str">
-        <v>Anthropic</v>
+        <v>Palo Alto Networks</v>
       </c>
       <c r="C12" t="str">
-        <v>Full Stack AI Engineer</v>
+        <v>OT Cybersecurity &amp; Threat Detection Engineer</v>
       </c>
       <c r="D12" t="str">
-        <v>Remote</v>
+        <v>Remote / Bengaluru</v>
       </c>
       <c r="E12" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F12" t="str">
-        <v>45%</v>
+        <v>61%</v>
       </c>
       <c r="G12" t="str">
         <v>Skipped</v>
@@ -860,24 +860,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K12" t="str">
-        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
+        <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
       </c>
       <c r="L12" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 61% below threshold (70%).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>app_1790008945002_1</v>
+        <v>app_1790009257131_1</v>
       </c>
       <c r="B13" t="str">
-        <v>Vercel</v>
+        <v>CrowdStrike</v>
       </c>
       <c r="C13" t="str">
-        <v>Frontend Cloud Infrastructure Engineer</v>
+        <v>AI Security &amp; Anomaly Analytics Specialist</v>
       </c>
       <c r="D13" t="str">
         <v>Remote</v>
@@ -886,7 +886,7 @@
         <v>Lever</v>
       </c>
       <c r="F13" t="str">
-        <v>45%</v>
+        <v>61%</v>
       </c>
       <c r="G13" t="str">
         <v>Skipped</v>
@@ -898,33 +898,33 @@
         <v>2026-09-21</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K13" t="str">
-        <v>https://vercel.com/careers/frontend-infrastructure</v>
+        <v>https://crowdstrike.com/careers/ai-security-specialist</v>
       </c>
       <c r="L13" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 61% below threshold (70%).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>app_1790008945002_2</v>
+        <v>app_1790009257131_2</v>
       </c>
       <c r="B14" t="str">
-        <v>Shopify</v>
+        <v>Darktrace</v>
       </c>
       <c r="C14" t="str">
-        <v>Senior React &amp; Node Developer</v>
+        <v>Cyber AI SOC Analyst</v>
       </c>
       <c r="D14" t="str">
-        <v>Remote</v>
+        <v>Remote / Hybrid</v>
       </c>
       <c r="E14" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F14" t="str">
-        <v>45%</v>
+        <v>50%</v>
       </c>
       <c r="G14" t="str">
         <v>Skipped</v>
@@ -936,24 +936,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J14" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K14" t="str">
-        <v>https://shopify.com/careers/react-node-dev</v>
+        <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
       </c>
       <c r="L14" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 50% below threshold (70%).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>app_1790008945003_3</v>
+        <v>app_1790009257131_3</v>
       </c>
       <c r="B15" t="str">
         <v>Cloudflare</v>
       </c>
       <c r="C15" t="str">
-        <v>Web Platform Security Engineer</v>
+        <v>Security Automation Engineer</v>
       </c>
       <c r="D15" t="str">
         <v>Remote</v>
@@ -962,7 +962,7 @@
         <v>Workday</v>
       </c>
       <c r="F15" t="str">
-        <v>45%</v>
+        <v>51%</v>
       </c>
       <c r="G15" t="str">
         <v>Skipped</v>
@@ -974,24 +974,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J15" t="str">
-        <v>2026-09-21T16:42:25.003Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K15" t="str">
-        <v>https://cloudflare.com/careers/web-security-engineer</v>
+        <v>https://cloudflare.com/careers/security-automation</v>
       </c>
       <c r="L15" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 51% below threshold (70%).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>app_1790008562109_0</v>
+        <v>app_1790009257131_4</v>
       </c>
       <c r="B16" t="str">
         <v>Anthropic</v>
       </c>
       <c r="C16" t="str">
-        <v>Full Stack AI Engineer</v>
+        <v>Full Stack AI Security Engineer</v>
       </c>
       <c r="D16" t="str">
         <v>Remote</v>
@@ -1000,45 +1000,45 @@
         <v>Greenhouse</v>
       </c>
       <c r="F16" t="str">
-        <v>75%</v>
+        <v>50%</v>
       </c>
       <c r="G16" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H16" t="str">
-        <v>Under Review</v>
+        <v>Skipped</v>
       </c>
       <c r="I16" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J16" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K16" t="str">
-        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
+        <v>https://anthropic.com/careers/fullstack-ai-security</v>
       </c>
       <c r="L16" t="str">
-        <v>Auto-filled profile data for Karthikeyan R.</v>
+        <v>Skipped: Match score 50% below threshold (70%).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>app_1790008562109_1</v>
+        <v>app_1790008945002_0</v>
       </c>
       <c r="B17" t="str">
-        <v>Vercel</v>
+        <v>Anthropic</v>
       </c>
       <c r="C17" t="str">
-        <v>Frontend Cloud Infrastructure Engineer</v>
+        <v>Full Stack AI Engineer</v>
       </c>
       <c r="D17" t="str">
         <v>Remote</v>
       </c>
       <c r="E17" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F17" t="str">
-        <v>53%</v>
+        <v>45%</v>
       </c>
       <c r="G17" t="str">
         <v>Skipped</v>
@@ -1050,33 +1050,33 @@
         <v>2026-09-21</v>
       </c>
       <c r="J17" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K17" t="str">
-        <v>https://vercel.com/careers/frontend-infrastructure</v>
+        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
       </c>
       <c r="L17" t="str">
-        <v>Skipped: Match score 53% below configured minimum (70%).</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>app_1790008562109_2</v>
+        <v>app_1790008945002_1</v>
       </c>
       <c r="B18" t="str">
-        <v>Shopify</v>
+        <v>Vercel</v>
       </c>
       <c r="C18" t="str">
-        <v>Senior React &amp; Node Developer</v>
+        <v>Frontend Cloud Infrastructure Engineer</v>
       </c>
       <c r="D18" t="str">
         <v>Remote</v>
       </c>
       <c r="E18" t="str">
-        <v>Greenhouse</v>
+        <v>Lever</v>
       </c>
       <c r="F18" t="str">
-        <v>53%</v>
+        <v>45%</v>
       </c>
       <c r="G18" t="str">
         <v>Skipped</v>
@@ -1088,30 +1088,30 @@
         <v>2026-09-21</v>
       </c>
       <c r="J18" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K18" t="str">
-        <v>https://shopify.com/careers/react-node-dev</v>
+        <v>https://vercel.com/careers/frontend-infrastructure</v>
       </c>
       <c r="L18" t="str">
-        <v>Skipped: Match score 53% below configured minimum (70%).</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>app_1790008562109_3</v>
+        <v>app_1790008945002_2</v>
       </c>
       <c r="B19" t="str">
-        <v>Cloudflare</v>
+        <v>Shopify</v>
       </c>
       <c r="C19" t="str">
-        <v>Web Platform Security Engineer</v>
+        <v>Senior React &amp; Node Developer</v>
       </c>
       <c r="D19" t="str">
         <v>Remote</v>
       </c>
       <c r="E19" t="str">
-        <v>Workday</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F19" t="str">
         <v>45%</v>
@@ -1126,10 +1126,10 @@
         <v>2026-09-21</v>
       </c>
       <c r="J19" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K19" t="str">
-        <v>https://cloudflare.com/careers/web-security-engineer</v>
+        <v>https://shopify.com/careers/react-node-dev</v>
       </c>
       <c r="L19" t="str">
         <v>Skipped: Match score 45% below configured minimum (70%).</v>
@@ -1137,60 +1137,60 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>app_1001</v>
+        <v>app_1790008945003_3</v>
       </c>
       <c r="B20" t="str">
-        <v>Vercel</v>
+        <v>Cloudflare</v>
       </c>
       <c r="C20" t="str">
-        <v>Senior Frontend Engineer - React</v>
+        <v>Web Platform Security Engineer</v>
       </c>
       <c r="D20" t="str">
         <v>Remote</v>
       </c>
       <c r="E20" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F20" t="str">
-        <v>94%</v>
+        <v>45%</v>
       </c>
       <c r="G20" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H20" t="str">
-        <v>Interview Scheduled</v>
+        <v>Skipped</v>
       </c>
       <c r="I20" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J20" t="str">
-        <v>2026-09-21T09:12:00Z</v>
+        <v>2026-09-21T16:42:25.003Z</v>
       </c>
       <c r="K20" t="str">
-        <v>https://vercel.com/careers/senior-frontend-engineer</v>
+        <v>https://cloudflare.com/careers/web-security-engineer</v>
       </c>
       <c r="L20" t="str">
-        <v>Submitted with custom cover letter &amp; React portfolio link.</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>app_1002</v>
+        <v>app_1790008562109_0</v>
       </c>
       <c r="B21" t="str">
-        <v>Stripe</v>
+        <v>Anthropic</v>
       </c>
       <c r="C21" t="str">
-        <v>Full Stack Engineer - Developer Experience</v>
+        <v>Full Stack AI Engineer</v>
       </c>
       <c r="D21" t="str">
-        <v>Remote (US/Global)</v>
+        <v>Remote</v>
       </c>
       <c r="E21" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F21" t="str">
-        <v>91%</v>
+        <v>75%</v>
       </c>
       <c r="G21" t="str">
         <v>Applied</v>
@@ -1202,24 +1202,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J21" t="str">
-        <v>2026-09-21T09:18:22Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K21" t="str">
-        <v>https://stripe.com/jobs/full-stack-dx</v>
+        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
       </c>
       <c r="L21" t="str">
-        <v>Auto-filled standard Q&amp;A. Verified 4+ yrs React/Node experience.</v>
+        <v>Auto-filled profile data for Karthikeyan R.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>app_1003</v>
+        <v>app_1790008562109_1</v>
       </c>
       <c r="B22" t="str">
-        <v>Supabase</v>
+        <v>Vercel</v>
       </c>
       <c r="C22" t="str">
-        <v>Full Stack Developer (Next.js &amp; Postgres)</v>
+        <v>Frontend Cloud Infrastructure Engineer</v>
       </c>
       <c r="D22" t="str">
         <v>Remote</v>
@@ -1228,159 +1228,159 @@
         <v>Lever</v>
       </c>
       <c r="F22" t="str">
-        <v>88%</v>
+        <v>53%</v>
       </c>
       <c r="G22" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H22" t="str">
-        <v>Under Review</v>
+        <v>Skipped</v>
       </c>
       <c r="I22" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J22" t="str">
-        <v>2026-09-21T09:24:10Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K22" t="str">
-        <v>https://supabase.com/careers/full-stack-dev</v>
+        <v>https://vercel.com/careers/frontend-infrastructure</v>
       </c>
       <c r="L22" t="str">
-        <v>Matched skills: PostgreSQL, React, TypeScript, FastAPI.</v>
+        <v>Skipped: Match score 53% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>app_1004</v>
+        <v>app_1790008562109_2</v>
       </c>
       <c r="B23" t="str">
-        <v>Linear</v>
+        <v>Shopify</v>
       </c>
       <c r="C23" t="str">
-        <v>Frontend Architect</v>
+        <v>Senior React &amp; Node Developer</v>
       </c>
       <c r="D23" t="str">
-        <v>Remote / San Francisco</v>
+        <v>Remote</v>
       </c>
       <c r="E23" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F23" t="str">
-        <v>76%</v>
+        <v>53%</v>
       </c>
       <c r="G23" t="str">
-        <v>Review Required</v>
+        <v>Skipped</v>
       </c>
       <c r="H23" t="str">
-        <v>Action Needed</v>
+        <v>Skipped</v>
       </c>
       <c r="I23" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J23" t="str">
-        <v>2026-09-21T09:30:45Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K23" t="str">
-        <v>https://linear.app/careers/frontend-architect</v>
+        <v>https://shopify.com/careers/react-node-dev</v>
       </c>
       <c r="L23" t="str">
-        <v>Form requires custom video introduction URL. Paused for user input.</v>
+        <v>Skipped: Match score 53% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>app_1005</v>
+        <v>app_1790008562109_3</v>
       </c>
       <c r="B24" t="str">
-        <v>OpenAI</v>
+        <v>Cloudflare</v>
       </c>
       <c r="C24" t="str">
-        <v>AI Applications Engineer</v>
+        <v>Web Platform Security Engineer</v>
       </c>
       <c r="D24" t="str">
-        <v>Remote / Hybrid</v>
+        <v>Remote</v>
       </c>
       <c r="E24" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F24" t="str">
-        <v>96%</v>
+        <v>45%</v>
       </c>
       <c r="G24" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H24" t="str">
-        <v>Screening Call</v>
+        <v>Skipped</v>
       </c>
       <c r="I24" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J24" t="str">
-        <v>2026-09-21T09:35:12Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K24" t="str">
-        <v>https://openai.com/careers/ai-applications-engineer</v>
+        <v>https://cloudflare.com/careers/web-security-engineer</v>
       </c>
       <c r="L24" t="str">
-        <v>High match score! Highlighted LLM integration &amp; FastAPI projects.</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>app_0995</v>
+        <v>app_1001</v>
       </c>
       <c r="B25" t="str">
-        <v>Postman</v>
+        <v>Vercel</v>
       </c>
       <c r="C25" t="str">
-        <v>Full Stack Engineer - API Network</v>
+        <v>Senior Frontend Engineer - React</v>
       </c>
       <c r="D25" t="str">
-        <v>Bengaluru (Hybrid)</v>
+        <v>Remote</v>
       </c>
       <c r="E25" t="str">
-        <v>Workday</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F25" t="str">
-        <v>89%</v>
+        <v>94%</v>
       </c>
       <c r="G25" t="str">
         <v>Applied</v>
       </c>
       <c r="H25" t="str">
-        <v>Assessment Sent</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I25" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J25" t="str">
-        <v>2026-09-20T09:05:00Z</v>
+        <v>2026-09-21T09:12:00Z</v>
       </c>
       <c r="K25" t="str">
-        <v>https://postman.com/careers/fullstack-eng</v>
+        <v>https://vercel.com/careers/senior-frontend-engineer</v>
       </c>
       <c r="L25" t="str">
-        <v>Applied via automated profile submitter.</v>
+        <v>Submitted with custom cover letter &amp; React portfolio link.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>app_0996</v>
+        <v>app_1002</v>
       </c>
       <c r="B26" t="str">
-        <v>Datadog</v>
+        <v>Stripe</v>
       </c>
       <c r="C26" t="str">
-        <v>Software Engineer - UI Dashboards</v>
+        <v>Full Stack Engineer - Developer Experience</v>
       </c>
       <c r="D26" t="str">
-        <v>Remote</v>
+        <v>Remote (US/Global)</v>
       </c>
       <c r="E26" t="str">
-        <v>Greenhouse</v>
+        <v>Lever</v>
       </c>
       <c r="F26" t="str">
-        <v>85%</v>
+        <v>91%</v>
       </c>
       <c r="G26" t="str">
         <v>Applied</v>
@@ -1389,27 +1389,27 @@
         <v>Under Review</v>
       </c>
       <c r="I26" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J26" t="str">
-        <v>2026-09-20T09:14:30Z</v>
+        <v>2026-09-21T09:18:22Z</v>
       </c>
       <c r="K26" t="str">
-        <v>https://datadog.com/careers/ui-engineer</v>
+        <v>https://stripe.com/jobs/full-stack-dx</v>
       </c>
       <c r="L26" t="str">
-        <v>Form submission successful.</v>
+        <v>Auto-filled standard Q&amp;A. Verified 4+ yrs React/Node experience.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>app_0997</v>
+        <v>app_1003</v>
       </c>
       <c r="B27" t="str">
-        <v>Figma</v>
+        <v>Supabase</v>
       </c>
       <c r="C27" t="str">
-        <v>Design Systems Developer</v>
+        <v>Full Stack Developer (Next.js &amp; Postgres)</v>
       </c>
       <c r="D27" t="str">
         <v>Remote</v>
@@ -1418,7 +1418,7 @@
         <v>Lever</v>
       </c>
       <c r="F27" t="str">
-        <v>82%</v>
+        <v>88%</v>
       </c>
       <c r="G27" t="str">
         <v>Applied</v>
@@ -1427,173 +1427,363 @@
         <v>Under Review</v>
       </c>
       <c r="I27" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J27" t="str">
-        <v>2026-09-20T09:22:15Z</v>
+        <v>2026-09-21T09:24:10Z</v>
       </c>
       <c r="K27" t="str">
-        <v>https://figma.com/careers/design-systems-dev</v>
+        <v>https://supabase.com/careers/full-stack-dev</v>
       </c>
       <c r="L27" t="str">
-        <v>Attached CSS/React portfolio link.</v>
+        <v>Matched skills: PostgreSQL, React, TypeScript, FastAPI.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>app_0998</v>
+        <v>app_1004</v>
       </c>
       <c r="B28" t="str">
-        <v>Notion</v>
+        <v>Linear</v>
       </c>
       <c r="C28" t="str">
-        <v>Product Engineer - Workspace</v>
+        <v>Frontend Architect</v>
       </c>
       <c r="D28" t="str">
-        <v>Remote</v>
+        <v>Remote / San Francisco</v>
       </c>
       <c r="E28" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F28" t="str">
-        <v>68%</v>
+        <v>76%</v>
       </c>
       <c r="G28" t="str">
-        <v>Skipped</v>
+        <v>Review Required</v>
       </c>
       <c r="H28" t="str">
-        <v>Skipped</v>
+        <v>Action Needed</v>
       </c>
       <c r="I28" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J28" t="str">
-        <v>2026-09-20T09:28:00Z</v>
+        <v>2026-09-21T09:30:45Z</v>
       </c>
       <c r="K28" t="str">
-        <v>https://notion.so/careers/product-engineer</v>
+        <v>https://linear.app/careers/frontend-architect</v>
       </c>
       <c r="L28" t="str">
-        <v>Skipped: Match score 68% below threshold minimum 70%.</v>
+        <v>Form requires custom video introduction URL. Paused for user input.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>app_0988</v>
+        <v>app_1005</v>
       </c>
       <c r="B29" t="str">
-        <v>Razorpay</v>
+        <v>OpenAI</v>
       </c>
       <c r="C29" t="str">
-        <v>Senior Frontend Developer</v>
+        <v>AI Applications Engineer</v>
       </c>
       <c r="D29" t="str">
-        <v>Bengaluru</v>
+        <v>Remote / Hybrid</v>
       </c>
       <c r="E29" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F29" t="str">
-        <v>92%</v>
+        <v>96%</v>
       </c>
       <c r="G29" t="str">
         <v>Applied</v>
       </c>
       <c r="H29" t="str">
-        <v>Interview Scheduled</v>
+        <v>Screening Call</v>
       </c>
       <c r="I29" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J29" t="str">
-        <v>2026-09-19T09:10:00Z</v>
+        <v>2026-09-21T09:35:12Z</v>
       </c>
       <c r="K29" t="str">
-        <v>https://razorpay.com/careers/frontend-sr</v>
+        <v>https://openai.com/careers/ai-applications-engineer</v>
       </c>
       <c r="L29" t="str">
-        <v>Applied successfully.</v>
+        <v>High match score! Highlighted LLM integration &amp; FastAPI projects.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>app_0989</v>
+        <v>app_0995</v>
       </c>
       <c r="B30" t="str">
-        <v>GitHub</v>
+        <v>Postman</v>
       </c>
       <c r="C30" t="str">
-        <v>Software Engineer - Copilot Extensions</v>
+        <v>Full Stack Engineer - API Network</v>
       </c>
       <c r="D30" t="str">
-        <v>Remote</v>
+        <v>Bengaluru (Hybrid)</v>
       </c>
       <c r="E30" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F30" t="str">
-        <v>95%</v>
+        <v>89%</v>
       </c>
       <c r="G30" t="str">
         <v>Applied</v>
       </c>
       <c r="H30" t="str">
-        <v>Screening Call</v>
+        <v>Assessment Sent</v>
       </c>
       <c r="I30" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-20</v>
       </c>
       <c r="J30" t="str">
-        <v>2026-09-19T09:16:40Z</v>
+        <v>2026-09-20T09:05:00Z</v>
       </c>
       <c r="K30" t="str">
-        <v>https://github.com/careers/copilot-engineer</v>
+        <v>https://postman.com/careers/fullstack-eng</v>
       </c>
       <c r="L30" t="str">
-        <v>Matched AI &amp; extension development skills.</v>
+        <v>Applied via automated profile submitter.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>app_0996</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Datadog</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Software Engineer - UI Dashboards</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F31" t="str">
+        <v>85%</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Under Review</v>
+      </c>
+      <c r="I31" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J31" t="str">
+        <v>2026-09-20T09:14:30Z</v>
+      </c>
+      <c r="K31" t="str">
+        <v>https://datadog.com/careers/ui-engineer</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Form submission successful.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>app_0997</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Figma</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Design Systems Developer</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Lever</v>
+      </c>
+      <c r="F32" t="str">
+        <v>82%</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Under Review</v>
+      </c>
+      <c r="I32" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J32" t="str">
+        <v>2026-09-20T09:22:15Z</v>
+      </c>
+      <c r="K32" t="str">
+        <v>https://figma.com/careers/design-systems-dev</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Attached CSS/React portfolio link.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>app_0998</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Notion</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Product Engineer - Workspace</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Lever</v>
+      </c>
+      <c r="F33" t="str">
+        <v>68%</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="I33" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J33" t="str">
+        <v>2026-09-20T09:28:00Z</v>
+      </c>
+      <c r="K33" t="str">
+        <v>https://notion.so/careers/product-engineer</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Skipped: Match score 68% below threshold minimum 70%.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>app_0988</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Razorpay</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Senior Frontend Developer</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F34" t="str">
+        <v>92%</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="I34" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="J34" t="str">
+        <v>2026-09-19T09:10:00Z</v>
+      </c>
+      <c r="K34" t="str">
+        <v>https://razorpay.com/careers/frontend-sr</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Applied successfully.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>app_0989</v>
+      </c>
+      <c r="B35" t="str">
+        <v>GitHub</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Software Engineer - Copilot Extensions</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F35" t="str">
+        <v>95%</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Screening Call</v>
+      </c>
+      <c r="I35" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="J35" t="str">
+        <v>2026-09-19T09:16:40Z</v>
+      </c>
+      <c r="K35" t="str">
+        <v>https://github.com/careers/copilot-engineer</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Matched AI &amp; extension development skills.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>app_0980</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B36" t="str">
         <v>GitLab</v>
       </c>
-      <c r="C31" t="str">
+      <c r="C36" t="str">
         <v>Full Stack Engineer - AI Features</v>
       </c>
-      <c r="D31" t="str">
-        <v>Remote</v>
-      </c>
-      <c r="E31" t="str">
+      <c r="D36" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E36" t="str">
         <v>Lever</v>
       </c>
-      <c r="F31" t="str">
+      <c r="F36" t="str">
         <v>90%</v>
       </c>
-      <c r="G31" t="str">
-        <v>Applied</v>
-      </c>
-      <c r="H31" t="str">
+      <c r="G36" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H36" t="str">
         <v>Offer Received</v>
       </c>
-      <c r="I31" t="str">
+      <c r="I36" t="str">
         <v>2026-09-18</v>
       </c>
-      <c r="J31" t="str">
+      <c r="J36" t="str">
         <v>2026-09-18T09:05:10Z</v>
       </c>
-      <c r="K31" t="str">
+      <c r="K36" t="str">
         <v>https://gitlab.com/jobs/fullstack-ai</v>
       </c>
-      <c r="L31" t="str">
+      <c r="L36" t="str">
         <v>Submitted with candidate profile.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add live Playwright Chrome browser form automation & screenshot verification
</commit_message>
<xml_diff>
--- a/data/applications_tracker.xlsx
+++ b/data/applications_tracker.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L41"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -453,7 +453,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>app_1790010835509_0</v>
+        <v>app_1790013705404_0</v>
       </c>
       <c r="B2" t="str">
         <v>Palo Alto Networks</v>
@@ -480,7 +480,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-09-21T17:13:55.509Z</v>
+        <v>2026-09-21T18:01:45.404Z</v>
       </c>
       <c r="K2" t="str">
         <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
@@ -491,7 +491,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>app_1790010835509_1</v>
+        <v>app_1790013705405_1</v>
       </c>
       <c r="B3" t="str">
         <v>CrowdStrike</v>
@@ -518,7 +518,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-09-21T17:13:55.509Z</v>
+        <v>2026-09-21T18:01:45.405Z</v>
       </c>
       <c r="K3" t="str">
         <v>https://crowdstrike.com/careers/ai-security-specialist</v>
@@ -529,7 +529,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>app_1790010835510_2</v>
+        <v>app_1790013705405_2</v>
       </c>
       <c r="B4" t="str">
         <v>Darktrace</v>
@@ -556,7 +556,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-09-21T17:13:55.510Z</v>
+        <v>2026-09-21T18:01:45.405Z</v>
       </c>
       <c r="K4" t="str">
         <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>app_1790010835510_3</v>
+        <v>app_1790013705405_3</v>
       </c>
       <c r="B5" t="str">
         <v>Cloudflare</v>
@@ -594,7 +594,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-09-21T17:13:55.510Z</v>
+        <v>2026-09-21T18:01:45.405Z</v>
       </c>
       <c r="K5" t="str">
         <v>https://cloudflare.com/careers/security-automation</v>
@@ -605,7 +605,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>app_1790010835510_4</v>
+        <v>app_1790013705405_4</v>
       </c>
       <c r="B6" t="str">
         <v>Anthropic</v>
@@ -632,7 +632,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-09-21T17:13:55.510Z</v>
+        <v>2026-09-21T18:01:45.405Z</v>
       </c>
       <c r="K6" t="str">
         <v>https://anthropic.com/careers/fullstack-ai-security</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>app_1790009309416_0</v>
+        <v>app_1790010835509_0</v>
       </c>
       <c r="B7" t="str">
         <v>Palo Alto Networks</v>
@@ -670,7 +670,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.509Z</v>
       </c>
       <c r="K7" t="str">
         <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
@@ -681,7 +681,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>app_1790009309416_1</v>
+        <v>app_1790010835509_1</v>
       </c>
       <c r="B8" t="str">
         <v>CrowdStrike</v>
@@ -708,7 +708,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.509Z</v>
       </c>
       <c r="K8" t="str">
         <v>https://crowdstrike.com/careers/ai-security-specialist</v>
@@ -719,7 +719,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>app_1790009309416_2</v>
+        <v>app_1790010835510_2</v>
       </c>
       <c r="B9" t="str">
         <v>Darktrace</v>
@@ -746,7 +746,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J9" t="str">
-        <v>2026-09-21T16:48:29.416Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K9" t="str">
         <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
@@ -757,7 +757,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>app_1790009309417_3</v>
+        <v>app_1790010835510_3</v>
       </c>
       <c r="B10" t="str">
         <v>Cloudflare</v>
@@ -784,7 +784,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J10" t="str">
-        <v>2026-09-21T16:48:29.417Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K10" t="str">
         <v>https://cloudflare.com/careers/security-automation</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>app_1790009309417_4</v>
+        <v>app_1790010835510_4</v>
       </c>
       <c r="B11" t="str">
         <v>Anthropic</v>
@@ -822,7 +822,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="J11" t="str">
-        <v>2026-09-21T16:48:29.417Z</v>
+        <v>2026-09-21T17:13:55.510Z</v>
       </c>
       <c r="K11" t="str">
         <v>https://anthropic.com/careers/fullstack-ai-security</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>app_1790009257131_0</v>
+        <v>app_1790009309416_0</v>
       </c>
       <c r="B12" t="str">
         <v>Palo Alto Networks</v>
@@ -848,30 +848,30 @@
         <v>Greenhouse</v>
       </c>
       <c r="F12" t="str">
-        <v>61%</v>
+        <v>92%</v>
       </c>
       <c r="G12" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H12" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I12" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K12" t="str">
         <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
       </c>
       <c r="L12" t="str">
-        <v>Skipped: Match score 61% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>app_1790009257131_1</v>
+        <v>app_1790009309416_1</v>
       </c>
       <c r="B13" t="str">
         <v>CrowdStrike</v>
@@ -886,30 +886,30 @@
         <v>Lever</v>
       </c>
       <c r="F13" t="str">
-        <v>61%</v>
+        <v>92%</v>
       </c>
       <c r="G13" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H13" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I13" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K13" t="str">
         <v>https://crowdstrike.com/careers/ai-security-specialist</v>
       </c>
       <c r="L13" t="str">
-        <v>Skipped: Match score 61% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>app_1790009257131_2</v>
+        <v>app_1790009309416_2</v>
       </c>
       <c r="B14" t="str">
         <v>Darktrace</v>
@@ -924,30 +924,30 @@
         <v>Greenhouse</v>
       </c>
       <c r="F14" t="str">
-        <v>50%</v>
+        <v>74%</v>
       </c>
       <c r="G14" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H14" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I14" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J14" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.416Z</v>
       </c>
       <c r="K14" t="str">
         <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
       </c>
       <c r="L14" t="str">
-        <v>Skipped: Match score 50% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>app_1790009257131_3</v>
+        <v>app_1790009309417_3</v>
       </c>
       <c r="B15" t="str">
         <v>Cloudflare</v>
@@ -962,30 +962,30 @@
         <v>Workday</v>
       </c>
       <c r="F15" t="str">
-        <v>51%</v>
+        <v>90%</v>
       </c>
       <c r="G15" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H15" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I15" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J15" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.417Z</v>
       </c>
       <c r="K15" t="str">
         <v>https://cloudflare.com/careers/security-automation</v>
       </c>
       <c r="L15" t="str">
-        <v>Skipped: Match score 51% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>app_1790009257131_4</v>
+        <v>app_1790009309417_4</v>
       </c>
       <c r="B16" t="str">
         <v>Anthropic</v>
@@ -1000,45 +1000,45 @@
         <v>Greenhouse</v>
       </c>
       <c r="F16" t="str">
-        <v>50%</v>
+        <v>74%</v>
       </c>
       <c r="G16" t="str">
-        <v>Skipped</v>
+        <v>Applied</v>
       </c>
       <c r="H16" t="str">
-        <v>Skipped</v>
+        <v>Under Review</v>
       </c>
       <c r="I16" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J16" t="str">
-        <v>2026-09-21T16:47:37.131Z</v>
+        <v>2026-09-21T16:48:29.417Z</v>
       </c>
       <c r="K16" t="str">
         <v>https://anthropic.com/careers/fullstack-ai-security</v>
       </c>
       <c r="L16" t="str">
-        <v>Skipped: Match score 50% below threshold (70%).</v>
+        <v>Auto-filled profile data for M KARTHIKEYAN (PwC AI &amp; OT Security background).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>app_1790008945002_0</v>
+        <v>app_1790009257131_0</v>
       </c>
       <c r="B17" t="str">
-        <v>Anthropic</v>
+        <v>Palo Alto Networks</v>
       </c>
       <c r="C17" t="str">
-        <v>Full Stack AI Engineer</v>
+        <v>OT Cybersecurity &amp; Threat Detection Engineer</v>
       </c>
       <c r="D17" t="str">
-        <v>Remote</v>
+        <v>Remote / Bengaluru</v>
       </c>
       <c r="E17" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F17" t="str">
-        <v>45%</v>
+        <v>61%</v>
       </c>
       <c r="G17" t="str">
         <v>Skipped</v>
@@ -1050,24 +1050,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J17" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K17" t="str">
-        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
+        <v>https://paloaltonetworks.com/careers/ot-cybersecurity-engineer</v>
       </c>
       <c r="L17" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 61% below threshold (70%).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>app_1790008945002_1</v>
+        <v>app_1790009257131_1</v>
       </c>
       <c r="B18" t="str">
-        <v>Vercel</v>
+        <v>CrowdStrike</v>
       </c>
       <c r="C18" t="str">
-        <v>Frontend Cloud Infrastructure Engineer</v>
+        <v>AI Security &amp; Anomaly Analytics Specialist</v>
       </c>
       <c r="D18" t="str">
         <v>Remote</v>
@@ -1076,7 +1076,7 @@
         <v>Lever</v>
       </c>
       <c r="F18" t="str">
-        <v>45%</v>
+        <v>61%</v>
       </c>
       <c r="G18" t="str">
         <v>Skipped</v>
@@ -1088,33 +1088,33 @@
         <v>2026-09-21</v>
       </c>
       <c r="J18" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K18" t="str">
-        <v>https://vercel.com/careers/frontend-infrastructure</v>
+        <v>https://crowdstrike.com/careers/ai-security-specialist</v>
       </c>
       <c r="L18" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 61% below threshold (70%).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>app_1790008945002_2</v>
+        <v>app_1790009257131_2</v>
       </c>
       <c r="B19" t="str">
-        <v>Shopify</v>
+        <v>Darktrace</v>
       </c>
       <c r="C19" t="str">
-        <v>Senior React &amp; Node Developer</v>
+        <v>Cyber AI SOC Analyst</v>
       </c>
       <c r="D19" t="str">
-        <v>Remote</v>
+        <v>Remote / Hybrid</v>
       </c>
       <c r="E19" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F19" t="str">
-        <v>45%</v>
+        <v>50%</v>
       </c>
       <c r="G19" t="str">
         <v>Skipped</v>
@@ -1126,24 +1126,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J19" t="str">
-        <v>2026-09-21T16:42:25.002Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K19" t="str">
-        <v>https://shopify.com/careers/react-node-dev</v>
+        <v>https://darktrace.com/careers/cyber-ai-soc-analyst</v>
       </c>
       <c r="L19" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 50% below threshold (70%).</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>app_1790008945003_3</v>
+        <v>app_1790009257131_3</v>
       </c>
       <c r="B20" t="str">
         <v>Cloudflare</v>
       </c>
       <c r="C20" t="str">
-        <v>Web Platform Security Engineer</v>
+        <v>Security Automation Engineer</v>
       </c>
       <c r="D20" t="str">
         <v>Remote</v>
@@ -1152,7 +1152,7 @@
         <v>Workday</v>
       </c>
       <c r="F20" t="str">
-        <v>45%</v>
+        <v>51%</v>
       </c>
       <c r="G20" t="str">
         <v>Skipped</v>
@@ -1164,24 +1164,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J20" t="str">
-        <v>2026-09-21T16:42:25.003Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K20" t="str">
-        <v>https://cloudflare.com/careers/web-security-engineer</v>
+        <v>https://cloudflare.com/careers/security-automation</v>
       </c>
       <c r="L20" t="str">
-        <v>Skipped: Match score 45% below configured minimum (70%).</v>
+        <v>Skipped: Match score 51% below threshold (70%).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>app_1790008562109_0</v>
+        <v>app_1790009257131_4</v>
       </c>
       <c r="B21" t="str">
         <v>Anthropic</v>
       </c>
       <c r="C21" t="str">
-        <v>Full Stack AI Engineer</v>
+        <v>Full Stack AI Security Engineer</v>
       </c>
       <c r="D21" t="str">
         <v>Remote</v>
@@ -1190,45 +1190,45 @@
         <v>Greenhouse</v>
       </c>
       <c r="F21" t="str">
-        <v>75%</v>
+        <v>50%</v>
       </c>
       <c r="G21" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H21" t="str">
-        <v>Under Review</v>
+        <v>Skipped</v>
       </c>
       <c r="I21" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J21" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:47:37.131Z</v>
       </c>
       <c r="K21" t="str">
-        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
+        <v>https://anthropic.com/careers/fullstack-ai-security</v>
       </c>
       <c r="L21" t="str">
-        <v>Auto-filled profile data for Karthikeyan R.</v>
+        <v>Skipped: Match score 50% below threshold (70%).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>app_1790008562109_1</v>
+        <v>app_1790008945002_0</v>
       </c>
       <c r="B22" t="str">
-        <v>Vercel</v>
+        <v>Anthropic</v>
       </c>
       <c r="C22" t="str">
-        <v>Frontend Cloud Infrastructure Engineer</v>
+        <v>Full Stack AI Engineer</v>
       </c>
       <c r="D22" t="str">
         <v>Remote</v>
       </c>
       <c r="E22" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F22" t="str">
-        <v>53%</v>
+        <v>45%</v>
       </c>
       <c r="G22" t="str">
         <v>Skipped</v>
@@ -1240,33 +1240,33 @@
         <v>2026-09-21</v>
       </c>
       <c r="J22" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K22" t="str">
-        <v>https://vercel.com/careers/frontend-infrastructure</v>
+        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
       </c>
       <c r="L22" t="str">
-        <v>Skipped: Match score 53% below configured minimum (70%).</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>app_1790008562109_2</v>
+        <v>app_1790008945002_1</v>
       </c>
       <c r="B23" t="str">
-        <v>Shopify</v>
+        <v>Vercel</v>
       </c>
       <c r="C23" t="str">
-        <v>Senior React &amp; Node Developer</v>
+        <v>Frontend Cloud Infrastructure Engineer</v>
       </c>
       <c r="D23" t="str">
         <v>Remote</v>
       </c>
       <c r="E23" t="str">
-        <v>Greenhouse</v>
+        <v>Lever</v>
       </c>
       <c r="F23" t="str">
-        <v>53%</v>
+        <v>45%</v>
       </c>
       <c r="G23" t="str">
         <v>Skipped</v>
@@ -1278,30 +1278,30 @@
         <v>2026-09-21</v>
       </c>
       <c r="J23" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K23" t="str">
-        <v>https://shopify.com/careers/react-node-dev</v>
+        <v>https://vercel.com/careers/frontend-infrastructure</v>
       </c>
       <c r="L23" t="str">
-        <v>Skipped: Match score 53% below configured minimum (70%).</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>app_1790008562109_3</v>
+        <v>app_1790008945002_2</v>
       </c>
       <c r="B24" t="str">
-        <v>Cloudflare</v>
+        <v>Shopify</v>
       </c>
       <c r="C24" t="str">
-        <v>Web Platform Security Engineer</v>
+        <v>Senior React &amp; Node Developer</v>
       </c>
       <c r="D24" t="str">
         <v>Remote</v>
       </c>
       <c r="E24" t="str">
-        <v>Workday</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F24" t="str">
         <v>45%</v>
@@ -1316,10 +1316,10 @@
         <v>2026-09-21</v>
       </c>
       <c r="J24" t="str">
-        <v>2026-09-21T16:36:02.109Z</v>
+        <v>2026-09-21T16:42:25.002Z</v>
       </c>
       <c r="K24" t="str">
-        <v>https://cloudflare.com/careers/web-security-engineer</v>
+        <v>https://shopify.com/careers/react-node-dev</v>
       </c>
       <c r="L24" t="str">
         <v>Skipped: Match score 45% below configured minimum (70%).</v>
@@ -1327,60 +1327,60 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>app_1001</v>
+        <v>app_1790008945003_3</v>
       </c>
       <c r="B25" t="str">
-        <v>Vercel</v>
+        <v>Cloudflare</v>
       </c>
       <c r="C25" t="str">
-        <v>Senior Frontend Engineer - React</v>
+        <v>Web Platform Security Engineer</v>
       </c>
       <c r="D25" t="str">
         <v>Remote</v>
       </c>
       <c r="E25" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F25" t="str">
-        <v>94%</v>
+        <v>45%</v>
       </c>
       <c r="G25" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H25" t="str">
-        <v>Interview Scheduled</v>
+        <v>Skipped</v>
       </c>
       <c r="I25" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J25" t="str">
-        <v>2026-09-21T09:12:00Z</v>
+        <v>2026-09-21T16:42:25.003Z</v>
       </c>
       <c r="K25" t="str">
-        <v>https://vercel.com/careers/senior-frontend-engineer</v>
+        <v>https://cloudflare.com/careers/web-security-engineer</v>
       </c>
       <c r="L25" t="str">
-        <v>Submitted with custom cover letter &amp; React portfolio link.</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>app_1002</v>
+        <v>app_1790008562109_0</v>
       </c>
       <c r="B26" t="str">
-        <v>Stripe</v>
+        <v>Anthropic</v>
       </c>
       <c r="C26" t="str">
-        <v>Full Stack Engineer - Developer Experience</v>
+        <v>Full Stack AI Engineer</v>
       </c>
       <c r="D26" t="str">
-        <v>Remote (US/Global)</v>
+        <v>Remote</v>
       </c>
       <c r="E26" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F26" t="str">
-        <v>91%</v>
+        <v>75%</v>
       </c>
       <c r="G26" t="str">
         <v>Applied</v>
@@ -1392,24 +1392,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="J26" t="str">
-        <v>2026-09-21T09:18:22Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K26" t="str">
-        <v>https://stripe.com/jobs/full-stack-dx</v>
+        <v>https://anthropic.com/careers/fullstack-ai-engineer</v>
       </c>
       <c r="L26" t="str">
-        <v>Auto-filled standard Q&amp;A. Verified 4+ yrs React/Node experience.</v>
+        <v>Auto-filled profile data for Karthikeyan R.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>app_1003</v>
+        <v>app_1790008562109_1</v>
       </c>
       <c r="B27" t="str">
-        <v>Supabase</v>
+        <v>Vercel</v>
       </c>
       <c r="C27" t="str">
-        <v>Full Stack Developer (Next.js &amp; Postgres)</v>
+        <v>Frontend Cloud Infrastructure Engineer</v>
       </c>
       <c r="D27" t="str">
         <v>Remote</v>
@@ -1418,159 +1418,159 @@
         <v>Lever</v>
       </c>
       <c r="F27" t="str">
-        <v>88%</v>
+        <v>53%</v>
       </c>
       <c r="G27" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H27" t="str">
-        <v>Under Review</v>
+        <v>Skipped</v>
       </c>
       <c r="I27" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J27" t="str">
-        <v>2026-09-21T09:24:10Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K27" t="str">
-        <v>https://supabase.com/careers/full-stack-dev</v>
+        <v>https://vercel.com/careers/frontend-infrastructure</v>
       </c>
       <c r="L27" t="str">
-        <v>Matched skills: PostgreSQL, React, TypeScript, FastAPI.</v>
+        <v>Skipped: Match score 53% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>app_1004</v>
+        <v>app_1790008562109_2</v>
       </c>
       <c r="B28" t="str">
-        <v>Linear</v>
+        <v>Shopify</v>
       </c>
       <c r="C28" t="str">
-        <v>Frontend Architect</v>
+        <v>Senior React &amp; Node Developer</v>
       </c>
       <c r="D28" t="str">
-        <v>Remote / San Francisco</v>
+        <v>Remote</v>
       </c>
       <c r="E28" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F28" t="str">
-        <v>76%</v>
+        <v>53%</v>
       </c>
       <c r="G28" t="str">
-        <v>Review Required</v>
+        <v>Skipped</v>
       </c>
       <c r="H28" t="str">
-        <v>Action Needed</v>
+        <v>Skipped</v>
       </c>
       <c r="I28" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J28" t="str">
-        <v>2026-09-21T09:30:45Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K28" t="str">
-        <v>https://linear.app/careers/frontend-architect</v>
+        <v>https://shopify.com/careers/react-node-dev</v>
       </c>
       <c r="L28" t="str">
-        <v>Form requires custom video introduction URL. Paused for user input.</v>
+        <v>Skipped: Match score 53% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>app_1005</v>
+        <v>app_1790008562109_3</v>
       </c>
       <c r="B29" t="str">
-        <v>OpenAI</v>
+        <v>Cloudflare</v>
       </c>
       <c r="C29" t="str">
-        <v>AI Applications Engineer</v>
+        <v>Web Platform Security Engineer</v>
       </c>
       <c r="D29" t="str">
-        <v>Remote / Hybrid</v>
+        <v>Remote</v>
       </c>
       <c r="E29" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F29" t="str">
-        <v>96%</v>
+        <v>45%</v>
       </c>
       <c r="G29" t="str">
-        <v>Applied</v>
+        <v>Skipped</v>
       </c>
       <c r="H29" t="str">
-        <v>Screening Call</v>
+        <v>Skipped</v>
       </c>
       <c r="I29" t="str">
         <v>2026-09-21</v>
       </c>
       <c r="J29" t="str">
-        <v>2026-09-21T09:35:12Z</v>
+        <v>2026-09-21T16:36:02.109Z</v>
       </c>
       <c r="K29" t="str">
-        <v>https://openai.com/careers/ai-applications-engineer</v>
+        <v>https://cloudflare.com/careers/web-security-engineer</v>
       </c>
       <c r="L29" t="str">
-        <v>High match score! Highlighted LLM integration &amp; FastAPI projects.</v>
+        <v>Skipped: Match score 45% below configured minimum (70%).</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>app_0995</v>
+        <v>app_1001</v>
       </c>
       <c r="B30" t="str">
-        <v>Postman</v>
+        <v>Vercel</v>
       </c>
       <c r="C30" t="str">
-        <v>Full Stack Engineer - API Network</v>
+        <v>Senior Frontend Engineer - React</v>
       </c>
       <c r="D30" t="str">
-        <v>Bengaluru (Hybrid)</v>
+        <v>Remote</v>
       </c>
       <c r="E30" t="str">
-        <v>Workday</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F30" t="str">
-        <v>89%</v>
+        <v>94%</v>
       </c>
       <c r="G30" t="str">
         <v>Applied</v>
       </c>
       <c r="H30" t="str">
-        <v>Assessment Sent</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I30" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J30" t="str">
-        <v>2026-09-20T09:05:00Z</v>
+        <v>2026-09-21T09:12:00Z</v>
       </c>
       <c r="K30" t="str">
-        <v>https://postman.com/careers/fullstack-eng</v>
+        <v>https://vercel.com/careers/senior-frontend-engineer</v>
       </c>
       <c r="L30" t="str">
-        <v>Applied via automated profile submitter.</v>
+        <v>Submitted with custom cover letter &amp; React portfolio link.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>app_0996</v>
+        <v>app_1002</v>
       </c>
       <c r="B31" t="str">
-        <v>Datadog</v>
+        <v>Stripe</v>
       </c>
       <c r="C31" t="str">
-        <v>Software Engineer - UI Dashboards</v>
+        <v>Full Stack Engineer - Developer Experience</v>
       </c>
       <c r="D31" t="str">
-        <v>Remote</v>
+        <v>Remote (US/Global)</v>
       </c>
       <c r="E31" t="str">
-        <v>Greenhouse</v>
+        <v>Lever</v>
       </c>
       <c r="F31" t="str">
-        <v>85%</v>
+        <v>91%</v>
       </c>
       <c r="G31" t="str">
         <v>Applied</v>
@@ -1579,27 +1579,27 @@
         <v>Under Review</v>
       </c>
       <c r="I31" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J31" t="str">
-        <v>2026-09-20T09:14:30Z</v>
+        <v>2026-09-21T09:18:22Z</v>
       </c>
       <c r="K31" t="str">
-        <v>https://datadog.com/careers/ui-engineer</v>
+        <v>https://stripe.com/jobs/full-stack-dx</v>
       </c>
       <c r="L31" t="str">
-        <v>Form submission successful.</v>
+        <v>Auto-filled standard Q&amp;A. Verified 4+ yrs React/Node experience.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>app_0997</v>
+        <v>app_1003</v>
       </c>
       <c r="B32" t="str">
-        <v>Figma</v>
+        <v>Supabase</v>
       </c>
       <c r="C32" t="str">
-        <v>Design Systems Developer</v>
+        <v>Full Stack Developer (Next.js &amp; Postgres)</v>
       </c>
       <c r="D32" t="str">
         <v>Remote</v>
@@ -1608,7 +1608,7 @@
         <v>Lever</v>
       </c>
       <c r="F32" t="str">
-        <v>82%</v>
+        <v>88%</v>
       </c>
       <c r="G32" t="str">
         <v>Applied</v>
@@ -1617,173 +1617,363 @@
         <v>Under Review</v>
       </c>
       <c r="I32" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J32" t="str">
-        <v>2026-09-20T09:22:15Z</v>
+        <v>2026-09-21T09:24:10Z</v>
       </c>
       <c r="K32" t="str">
-        <v>https://figma.com/careers/design-systems-dev</v>
+        <v>https://supabase.com/careers/full-stack-dev</v>
       </c>
       <c r="L32" t="str">
-        <v>Attached CSS/React portfolio link.</v>
+        <v>Matched skills: PostgreSQL, React, TypeScript, FastAPI.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>app_0998</v>
+        <v>app_1004</v>
       </c>
       <c r="B33" t="str">
-        <v>Notion</v>
+        <v>Linear</v>
       </c>
       <c r="C33" t="str">
-        <v>Product Engineer - Workspace</v>
+        <v>Frontend Architect</v>
       </c>
       <c r="D33" t="str">
-        <v>Remote</v>
+        <v>Remote / San Francisco</v>
       </c>
       <c r="E33" t="str">
-        <v>Lever</v>
+        <v>Greenhouse</v>
       </c>
       <c r="F33" t="str">
-        <v>68%</v>
+        <v>76%</v>
       </c>
       <c r="G33" t="str">
-        <v>Skipped</v>
+        <v>Review Required</v>
       </c>
       <c r="H33" t="str">
-        <v>Skipped</v>
+        <v>Action Needed</v>
       </c>
       <c r="I33" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J33" t="str">
-        <v>2026-09-20T09:28:00Z</v>
+        <v>2026-09-21T09:30:45Z</v>
       </c>
       <c r="K33" t="str">
-        <v>https://notion.so/careers/product-engineer</v>
+        <v>https://linear.app/careers/frontend-architect</v>
       </c>
       <c r="L33" t="str">
-        <v>Skipped: Match score 68% below threshold minimum 70%.</v>
+        <v>Form requires custom video introduction URL. Paused for user input.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>app_0988</v>
+        <v>app_1005</v>
       </c>
       <c r="B34" t="str">
-        <v>Razorpay</v>
+        <v>OpenAI</v>
       </c>
       <c r="C34" t="str">
-        <v>Senior Frontend Developer</v>
+        <v>AI Applications Engineer</v>
       </c>
       <c r="D34" t="str">
-        <v>Bengaluru</v>
+        <v>Remote / Hybrid</v>
       </c>
       <c r="E34" t="str">
         <v>Greenhouse</v>
       </c>
       <c r="F34" t="str">
-        <v>92%</v>
+        <v>96%</v>
       </c>
       <c r="G34" t="str">
         <v>Applied</v>
       </c>
       <c r="H34" t="str">
-        <v>Interview Scheduled</v>
+        <v>Screening Call</v>
       </c>
       <c r="I34" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-21</v>
       </c>
       <c r="J34" t="str">
-        <v>2026-09-19T09:10:00Z</v>
+        <v>2026-09-21T09:35:12Z</v>
       </c>
       <c r="K34" t="str">
-        <v>https://razorpay.com/careers/frontend-sr</v>
+        <v>https://openai.com/careers/ai-applications-engineer</v>
       </c>
       <c r="L34" t="str">
-        <v>Applied successfully.</v>
+        <v>High match score! Highlighted LLM integration &amp; FastAPI projects.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>app_0989</v>
+        <v>app_0995</v>
       </c>
       <c r="B35" t="str">
-        <v>GitHub</v>
+        <v>Postman</v>
       </c>
       <c r="C35" t="str">
-        <v>Software Engineer - Copilot Extensions</v>
+        <v>Full Stack Engineer - API Network</v>
       </c>
       <c r="D35" t="str">
-        <v>Remote</v>
+        <v>Bengaluru (Hybrid)</v>
       </c>
       <c r="E35" t="str">
-        <v>Greenhouse</v>
+        <v>Workday</v>
       </c>
       <c r="F35" t="str">
-        <v>95%</v>
+        <v>89%</v>
       </c>
       <c r="G35" t="str">
         <v>Applied</v>
       </c>
       <c r="H35" t="str">
-        <v>Screening Call</v>
+        <v>Assessment Sent</v>
       </c>
       <c r="I35" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-20</v>
       </c>
       <c r="J35" t="str">
-        <v>2026-09-19T09:16:40Z</v>
+        <v>2026-09-20T09:05:00Z</v>
       </c>
       <c r="K35" t="str">
-        <v>https://github.com/careers/copilot-engineer</v>
+        <v>https://postman.com/careers/fullstack-eng</v>
       </c>
       <c r="L35" t="str">
-        <v>Matched AI &amp; extension development skills.</v>
+        <v>Applied via automated profile submitter.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>app_0996</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Datadog</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Software Engineer - UI Dashboards</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F36" t="str">
+        <v>85%</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Under Review</v>
+      </c>
+      <c r="I36" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J36" t="str">
+        <v>2026-09-20T09:14:30Z</v>
+      </c>
+      <c r="K36" t="str">
+        <v>https://datadog.com/careers/ui-engineer</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Form submission successful.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>app_0997</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Figma</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Design Systems Developer</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Lever</v>
+      </c>
+      <c r="F37" t="str">
+        <v>82%</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Under Review</v>
+      </c>
+      <c r="I37" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J37" t="str">
+        <v>2026-09-20T09:22:15Z</v>
+      </c>
+      <c r="K37" t="str">
+        <v>https://figma.com/careers/design-systems-dev</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Attached CSS/React portfolio link.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>app_0998</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Notion</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Product Engineer - Workspace</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Lever</v>
+      </c>
+      <c r="F38" t="str">
+        <v>68%</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Skipped</v>
+      </c>
+      <c r="I38" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="J38" t="str">
+        <v>2026-09-20T09:28:00Z</v>
+      </c>
+      <c r="K38" t="str">
+        <v>https://notion.so/careers/product-engineer</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Skipped: Match score 68% below threshold minimum 70%.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>app_0988</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Razorpay</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Senior Frontend Developer</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F39" t="str">
+        <v>92%</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Interview Scheduled</v>
+      </c>
+      <c r="I39" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="J39" t="str">
+        <v>2026-09-19T09:10:00Z</v>
+      </c>
+      <c r="K39" t="str">
+        <v>https://razorpay.com/careers/frontend-sr</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Applied successfully.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>app_0989</v>
+      </c>
+      <c r="B40" t="str">
+        <v>GitHub</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Software Engineer - Copilot Extensions</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Greenhouse</v>
+      </c>
+      <c r="F40" t="str">
+        <v>95%</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Screening Call</v>
+      </c>
+      <c r="I40" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="J40" t="str">
+        <v>2026-09-19T09:16:40Z</v>
+      </c>
+      <c r="K40" t="str">
+        <v>https://github.com/careers/copilot-engineer</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Matched AI &amp; extension development skills.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
         <v>app_0980</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B41" t="str">
         <v>GitLab</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C41" t="str">
         <v>Full Stack Engineer - AI Features</v>
       </c>
-      <c r="D36" t="str">
-        <v>Remote</v>
-      </c>
-      <c r="E36" t="str">
+      <c r="D41" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E41" t="str">
         <v>Lever</v>
       </c>
-      <c r="F36" t="str">
+      <c r="F41" t="str">
         <v>90%</v>
       </c>
-      <c r="G36" t="str">
-        <v>Applied</v>
-      </c>
-      <c r="H36" t="str">
+      <c r="G41" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="H41" t="str">
         <v>Offer Received</v>
       </c>
-      <c r="I36" t="str">
+      <c r="I41" t="str">
         <v>2026-09-18</v>
       </c>
-      <c r="J36" t="str">
+      <c r="J41" t="str">
         <v>2026-09-18T09:05:10Z</v>
       </c>
-      <c r="K36" t="str">
+      <c r="K41" t="str">
         <v>https://gitlab.com/jobs/fullstack-ai</v>
       </c>
-      <c r="L36" t="str">
+      <c r="L41" t="str">
         <v>Submitted with candidate profile.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>